<commit_message>
Update sanitized dataset and generated outputs
</commit_message>
<xml_diff>
--- a/data/Combined_Maintenance_Log_Cleaned.xlsx
+++ b/data/Combined_Maintenance_Log_Cleaned.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,8 +501,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>44581</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2022-01-20 00:00:00</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -572,13 +570,15 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|0|SSLM21005SK|2022-01-20</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|0|Machine_001|2022-01-20</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>44589</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2022-01-28 00:00:00</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -651,13 +651,15 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|1|SSLM21005SK|2022-01-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|1|Machine_001|2022-01-28</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>44706</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2022-05-25 00:00:00</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -720,13 +722,15 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|2|SSLM21010SR|2022-05-25</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|2|Machine_002|2022-05-25</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>44719</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022-06-07 00:00:00</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -792,13 +796,15 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|3|SSLM21013NR|2022-06-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|3|Machine_003|2022-06-07</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>44727</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2022-06-15 00:00:00</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -860,13 +866,15 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|4|SSLM21003SRA|2022-06-15</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|4|Machine_004|2022-06-15</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>44742</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2022-06-30 00:00:00</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -939,13 +947,15 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|5|SSST30001WSD|2022-06-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|5|Machine_005|2022-06-30</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>44761</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2022-07-19 00:00:00</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1013,13 +1023,15 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|6|SSLM13001NR|2022-07-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|6|Machine_006|2022-07-19</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>44761</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2022-07-19 00:00:00</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1086,7 +1098,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|7|ASDM6122|2022-07-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|7|Machine_007|2022-07-19</t>
         </is>
       </c>
     </row>
@@ -1162,14 +1174,15 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|8|SSST10001BO
-SSLM22002SR|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|8|Machine_008|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>44887</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2022-11-22 00:00:00</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1243,13 +1256,15 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|9|SSST32002TC|2022-11-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|9|Machine_009|2022-11-22</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>44887</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2022-11-22 00:00:00</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1326,13 +1341,15 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|10|SSLM|2022-11-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|10|Machine_010|2022-11-22</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>45033</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2023-04-17 00:00:00</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1399,13 +1416,15 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|11|SSST30001TC|2023-04-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|11|Machine_011|2023-04-17</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>45030</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2023-04-14 00:00:00</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1472,13 +1491,15 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|12|SSLM21010NR|2023-04-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|12|Machine_012|2023-04-14</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>45058</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2023-05-12 00:00:00</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1548,13 +1569,15 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|13|SSLM21012SR|2023-05-12</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|13|Machine_013|2023-05-12</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>45093</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2023-06-16 00:00:00</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1621,13 +1644,15 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|14|SSLM21008SRNS|2023-06-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|14|Machine_014|2023-06-16</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>45042</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023-04-26 00:00:00</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1710,16 +1735,15 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|15|SSLM21010NR
-SSLM21011NR
-SSLM22101NR
-SSLM22102NR|2023-04-26</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|15|Machine_015|2023-04-26</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>45112</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2023-07-05 00:00:00</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1790,16 +1814,15 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|16|SSLM21010NR
-SSLM21011NR
-SSLM22101NR
-SSLM22102NR|2023-07-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|16|Machine_015|2023-07-05</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>45113</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2023-07-06 00:00:00</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1875,13 +1898,15 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|17|SSST30002WSD|2023-07-06</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|17|Machine_016|2023-07-06</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>45126</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2023-07-19 00:00:00</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1966,13 +1991,15 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|18|SSLM21003NR|2023-07-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|18|Machine_017|2023-07-19</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>45184</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2023-09-15 00:00:00</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -2038,14 +2065,15 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|19|SSLM
-(VAS)|2023-09-15</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|19|Machine_018|2023-09-15</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>45249</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2023-11-19 00:00:00</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2118,13 +2146,15 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|20|SSLM21011NR|2023-11-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|20|Machine_019|2023-11-19</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>45400</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2024-04-18 00:00:00</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2199,13 +2229,15 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|21|SSST32003TC|2024-04-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|21|Machine_020|2024-04-18</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>45436</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2024-05-24 00:00:00</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2272,13 +2304,15 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|22|ASLM32002|2024-05-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|22|Machine_021|2024-05-24</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>45446</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2024-06-03 00:00:00</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2361,13 +2395,15 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|23|SSLM21010NR|2024-06-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|23|Machine_012|2024-06-03</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>45508</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2024-08-04 00:00:00</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2450,13 +2486,15 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|24|SSLM23001SR|2024-08-04</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|24|Machine_022|2024-08-04</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>45489</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2024-07-16 00:00:00</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2534,14 +2572,15 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|25|SSLM25001NR
-SSLM25002NR|2024-07-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|25|Machine_023|2024-07-16</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>45596</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2024-10-31 00:00:00</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2611,13 +2650,15 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|26|SSLM21019SR|2024-10-31</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|26|Machine_024|2024-10-31</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>45627</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-12-01 00:00:00</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2695,13 +2736,15 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|27|SSST20004ZC|2024-12-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|27|Machine_025|2024-12-01</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>45042</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2023-04-26 00:00:00</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2770,13 +2813,15 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|28|SSLM21010NR|2023-04-26</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|28|Machine_012|2023-04-26</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>45705</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-02-17 00:00:00</t>
+        </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2841,13 +2886,15 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|29|ASSH10002|2025-02-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|29|Machine_026|2025-02-17</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>45713</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-02-25 00:00:00</t>
+        </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2924,14 +2971,15 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|30|PVOT0931
-(SSLM)|2025-02-25</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|30|Machine_027|2025-02-25</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>45743</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-03-27 00:00:00</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -3011,13 +3059,15 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|31|SSLM21001SRNS|2025-03-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|31|Machine_028|2025-03-27</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>45749</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-04-02 00:00:00</t>
+        </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -3097,13 +3147,15 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|32|ASSH5108|2025-04-02</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|32|Machine_029|2025-04-02</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>45769</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:00:00</t>
+        </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -3179,13 +3231,15 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|33|SSST20004TC|2025-04-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|33|Machine_030|2025-04-22</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>45782</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-05-05 00:00:00</t>
+        </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3263,13 +3317,15 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|34|SSLM25001NR|2025-05-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|34|Machine_031|2025-05-05</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>45866</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-07-28 00:00:00</t>
+        </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3345,13 +3401,15 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|35|SSST20001WCF|2025-07-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|35|Machine_032|2025-07-28</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>45884</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-08-15 00:00:00</t>
+        </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3424,13 +3482,15 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|36|SSLM21026SR|2025-08-15</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|36|Machine_033|2025-08-15</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>45896</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-08-27 00:00:00</t>
+        </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3501,13 +3561,15 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|37|SSLM21026SR|2025-08-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|37|Machine_033|2025-08-27</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>45898</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-08-29 00:00:00</t>
+        </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3586,13 +3648,15 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|38|SSLM21026SR|2025-08-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|38|Machine_033|2025-08-29</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>45904</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-09-04 00:00:00</t>
+        </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3670,13 +3734,15 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|39|SSST30003WSD|2025-09-04</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|39|Machine_034|2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>45928</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-09-28 00:00:00</t>
+        </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3745,13 +3811,15 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|40|SSST20003TS|2025-09-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|40|Machine_035|2025-09-28</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>45989</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-11-28 00:00:00</t>
+        </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3815,13 +3883,15 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|41|TTLM10015|2025-11-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|41|Machine_036|2025-11-28</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>46015</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-12-24 00:00:00</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3886,13 +3956,15 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|42|SSLM13011SR|2025-12-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|42|Machine_037|2025-12-24</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>46015</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-12-24 00:00:00</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3962,7 +4034,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|43|SSLM21001SRA|2025-12-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|軟體相關問題|43|Machine_038|2025-12-24</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4098,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -4039,13 +4111,15 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|0|SSLM21001SK|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|0|Machine_039|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>43592</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2019-05-07 00:00:00</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -4098,7 +4172,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -4111,13 +4185,15 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|1|SSST22001ZC|2019-05-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|1|Machine_040|2019-05-07</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>43593</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2019-05-08 00:00:00</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -4165,7 +4241,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -4178,13 +4254,15 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|2|SSST22001ZC|2019-05-08</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|2|Machine_040|2019-05-08</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>43594</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2019-05-09 00:00:00</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -4237,7 +4315,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -4250,13 +4328,15 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|3|SSLM13005NR|2019-05-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|3|Machine_041|2019-05-09</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>43606</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2019-05-21 00:00:00</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -4306,7 +4386,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -4319,13 +4399,15 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|4|SSLM21002SK|2019-05-21</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|4|Machine_042|2019-05-21</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>43608</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2019-05-23 00:00:00</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -4380,7 +4462,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4393,13 +4475,15 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|5|SSLM13006NR|2019-05-23</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|5|Machine_043|2019-05-23</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>43619</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2019-06-03 00:00:00</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -4448,7 +4532,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4461,7 +4545,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|6|SSLM11016SR|2019-06-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|6|Machine_044|2019-06-03</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4603,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4532,13 +4616,15 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|7|SSLM11016SR|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|7|Machine_044|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>43617</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2019-06-01 00:00:00</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -4595,7 +4681,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4608,13 +4694,15 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|8|SSLM21003SK|2019-06-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|8|Machine_045|2019-06-01</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>43627</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2019-06-11 00:00:00</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -4673,7 +4761,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4686,13 +4774,15 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|9|SSLM21003SK|2019-06-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|9|Machine_045|2019-06-11</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>43620</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2019-06-04 00:00:00</t>
+        </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -4745,7 +4835,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4758,7 +4848,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|10|SSLM21004SK|2019-06-04</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|10|Machine_046|2019-06-04</t>
         </is>
       </c>
     </row>
@@ -4820,7 +4910,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -4833,13 +4923,15 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|11|SSLM21004SK|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|11|Machine_046|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>43626</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2019-06-10 00:00:00</t>
+        </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -4892,7 +4984,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -4905,13 +4997,15 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|12|SSLM21004SK|2019-06-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|12|Machine_046|2019-06-10</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>43627</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2019-06-11 00:00:00</t>
+        </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4969,7 +5063,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -4982,13 +5076,15 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|13|SSLM21004SK|2019-06-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|13|Machine_046|2019-06-11</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>43629</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2019-06-13 00:00:00</t>
+        </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -5041,7 +5137,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -5054,13 +5150,15 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|14|SSLM11017SR|2019-06-13</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|14|Machine_047|2019-06-13</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>43626</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2019-06-10 00:00:00</t>
+        </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -5116,7 +5214,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -5129,7 +5227,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|15|SSST20006TC|2019-06-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|15|Machine_048|2019-06-10</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5289,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -5204,14 +5302,15 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|16|SSLM21003SK/
-SSLM21004SK|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|16|Machine_049|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>43739</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2019-10-01 00:00:00</t>
+        </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -5271,7 +5370,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -5284,13 +5383,15 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|17|SSLM21001SR|2019-10-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|17|Machine_050|2019-10-01</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>43754</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2019-10-16 00:00:00</t>
+        </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -5348,7 +5449,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -5361,13 +5462,15 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|18|SSLM21004NR|2019-10-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|18|Machine_051|2019-10-16</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>43757</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2019-10-19 00:00:00</t>
+        </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -5420,7 +5523,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5433,13 +5536,15 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|19|SSLM21001SK|2019-10-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|19|Machine_039|2019-10-19</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
-        <v>43770</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2019-11-01 00:00:00</t>
+        </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -5492,7 +5597,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -5505,13 +5610,15 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|20|SSLM21005SK|2019-11-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|20|Machine_001|2019-11-01</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
-        <v>43802</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2019-12-03 00:00:00</t>
+        </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -5564,7 +5671,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5577,13 +5684,15 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|21|TBPP11044|2019-12-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|21|Machine_052|2019-12-03</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
-        <v>43895</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2020-03-05 00:00:00</t>
+        </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -5637,7 +5746,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -5650,13 +5759,15 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|22|SSLM11018SR|2020-03-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|22|Machine_053|2020-03-05</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
-        <v>43903</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2020-03-13 00:00:00</t>
+        </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -5712,7 +5823,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -5725,13 +5836,15 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|23|SSST20001EE|2020-03-13</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|23|Machine_054|2020-03-13</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
-        <v>44048</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2020-08-05 00:00:00</t>
+        </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -5785,7 +5898,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -5798,13 +5911,15 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|24|SSLM21001NI|2020-08-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|24|Machine_055|2020-08-05</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
-        <v>44068</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2020-08-25 00:00:00</t>
+        </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5857,7 +5972,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -5870,13 +5985,15 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|25|SSLM21006NR|2020-08-25</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|25|Machine_056|2020-08-25</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
-        <v>44071</v>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2020-08-28 00:00:00</t>
+        </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -5937,7 +6054,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -5950,7 +6067,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|26|SSLM21006NR|2020-08-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|26|Machine_056|2020-08-28</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6139,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -6035,7 +6152,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|27|SSST22002TS|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|27|Machine_057|UNKNOWN</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6217,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -6113,13 +6230,15 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|28|SSLM22001SR|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|28|Machine_058|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>44284</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2021-03-29 00:00:00</t>
+        </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -6178,7 +6297,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -6191,13 +6310,15 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|29|SSLM13007SR|2021-03-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|29|Machine_059|2021-03-29</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
-        <v>44296</v>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2021-04-10 00:00:00</t>
+        </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -6251,7 +6372,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -6264,13 +6385,15 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|30|SSST22001TC|2021-04-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|30|Machine_060|2021-04-10</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
-        <v>44321</v>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2021-05-05 00:00:00</t>
+        </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -6329,7 +6452,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -6342,13 +6465,15 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|31|SSST22002TC|2021-05-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|31|Machine_061|2021-05-05</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
-        <v>44327</v>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2021-05-11 00:00:00</t>
+        </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -6403,7 +6528,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -6416,13 +6541,15 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|32|SSLM13008SR|2021-05-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|32|Machine_062|2021-05-11</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>44330</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2021-05-14 00:00:00</t>
+        </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -6471,7 +6598,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -6484,13 +6611,15 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|33|SSLM11022SR|2021-05-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|33|Machine_063|2021-05-14</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>44343</v>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2021-05-27 00:00:00</t>
+        </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -6540,7 +6669,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -6553,13 +6682,15 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|34|SSLM11023SR|2021-05-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|34|Machine_064|2021-05-27</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
-        <v>44396</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2021-07-19 00:00:00</t>
+        </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -6611,7 +6742,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -6624,13 +6755,15 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|35|SSST20001IC|2021-07-19</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|35|Machine_065|2021-07-19</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>44397</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2021-07-20 00:00:00</t>
+        </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -6702,7 +6835,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6715,13 +6848,15 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|36|SSST20001IC|2021-07-20</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|36|Machine_065|2021-07-20</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>44588</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2022-01-27 00:00:00</t>
+        </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -6777,7 +6912,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -6790,15 +6925,15 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|37|SSLM21022SR
-~
-SSLM21023SR|2022-01-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|37|Machine_066|2022-01-27</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>44588</v>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2022-01-27 00:00:00</t>
+        </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6857,7 +6992,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -6870,15 +7005,15 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|38|SSLM21021SR
-~
-SSLM21022SR|2022-01-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|38|Machine_067|2022-01-27</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>44599</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2022-02-07 00:00:00</t>
+        </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -6937,7 +7072,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6950,13 +7085,15 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|39|SSST20001ZC|2022-02-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|39|Machine_068|2022-02-07</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>44601</v>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2022-02-09 00:00:00</t>
+        </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -7020,7 +7157,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -7033,13 +7170,15 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|40|SSLM21023SR|2022-02-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|40|Machine_069|2022-02-09</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>44621</v>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2022-03-01 00:00:00</t>
+        </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -7095,7 +7234,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -7108,13 +7247,15 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|41|SSLM23001LRS|2022-03-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|41|Machine_070|2022-03-01</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>44629</v>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2022-03-09 00:00:00</t>
+        </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -7174,7 +7315,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -7187,13 +7328,15 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|42|SSLM21001SRNS|2022-03-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|42|Machine_028|2022-03-09</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>44650</v>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2022-03-30 00:00:00</t>
+        </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -7253,7 +7396,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -7266,14 +7409,15 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|43|SSST22001TSNS
-SSST22002TSNS|2022-03-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|43|Machine_071|2022-03-30</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>44650</v>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2022-03-30 00:00:00</t>
+        </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -7327,7 +7471,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -7340,8 +7484,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|44|SSST30003TS
-SSST20009TC|2022-03-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|44|Machine_072|2022-03-30</t>
         </is>
       </c>
     </row>
@@ -7412,7 +7555,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -7425,13 +7568,15 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|45|SSST30003TS|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|45|Machine_073|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
-        <v>44665</v>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2022-04-14 00:00:00</t>
+        </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -7487,7 +7632,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -7500,13 +7645,15 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|46|SSLM13013SR|2022-04-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|46|Machine_074|2022-04-14</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
-        <v>44679</v>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2022-04-28 00:00:00</t>
+        </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -7563,7 +7710,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -7576,13 +7723,15 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|47|SSST22002ZCS|2022-04-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|47|Machine_075|2022-04-28</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
-        <v>44679</v>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2022-04-28 00:00:00</t>
+        </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -7650,7 +7799,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -7663,13 +7812,15 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|48|SSST22002ZCS|2022-04-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|48|Machine_075|2022-04-28</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
-        <v>44680</v>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2022-04-29 00:00:00</t>
+        </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -7730,7 +7881,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -7743,13 +7894,15 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|49|SSLM21005SRNS|2022-04-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|49|Machine_076|2022-04-29</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
-        <v>44686</v>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2022-05-05 00:00:00</t>
+        </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -7807,7 +7960,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -7820,13 +7973,15 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|50|SSLM21005SRNS|2022-05-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|50|Machine_076|2022-05-05</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
-        <v>44707</v>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2022-05-26 00:00:00</t>
+        </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -7880,7 +8035,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -7893,13 +8048,15 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|51|SSST30002WSD|2022-05-26</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|51|Machine_016|2022-05-26</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
-        <v>44791</v>
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2022-08-18 00:00:00</t>
+        </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -7955,7 +8112,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7968,15 +8125,15 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|52|SSLM11029SR
-SSLM11030SR
-SSLM11031SR|2022-08-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|52|Machine_077|2022-08-18</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
-        <v>44791</v>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2022-08-18 00:00:00</t>
+        </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -8032,7 +8189,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -8045,15 +8202,15 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|53|SSST
-所有裝Ned的 
-分類機|2022-08-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|53|Machine_078|2022-08-18</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
-        <v>44887</v>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2022-11-22 00:00:00</t>
+        </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -8108,7 +8265,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -8121,13 +8278,15 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|54|SSST32002TC|2022-11-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|54|Machine_009|2022-11-22</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
-        <v>44895</v>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2022-11-30 00:00:00</t>
+        </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -8188,7 +8347,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -8201,8 +8360,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|55|SSST32002TC
-SSST32003TC|2022-11-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|55|Machine_079|2022-11-30</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8427,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -8282,14 +8440,15 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|56|TTLM20006
-TTLM20007|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|56|Machine_080|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
-        <v>45091</v>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2023-06-14 00:00:00</t>
+        </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8351,7 +8510,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -8364,13 +8523,15 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|57|FSLM21001KR|2023-06-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|57|Machine_081|2023-06-14</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
-        <v>45075</v>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2023-05-29 00:00:00</t>
+        </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8433,7 +8594,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -8446,13 +8607,15 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|58|SSST30003TS|2023-05-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|58|Machine_073|2023-05-29</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
-        <v>45159</v>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2023-08-21 00:00:00</t>
+        </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -8514,7 +8677,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -8527,13 +8690,15 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|59|SSLM21026SR|2023-08-21</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|59|Machine_033|2023-08-21</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
-        <v>45159</v>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2023-08-21 00:00:00</t>
+        </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -8592,7 +8757,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -8605,13 +8770,15 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|60|SSLM21029SR|2023-08-21</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|60|Machine_082|2023-08-21</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
-        <v>45159</v>
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2023-08-21 00:00:00</t>
+        </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -8671,7 +8838,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -8684,17 +8851,15 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|61|
-SSLM21026SR
-SSLM21027SR
-SSLM21028SR
-SSLM21029SR|2023-08-21</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|61|Machine_083|2023-08-21</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
-        <v>45167</v>
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2023-08-29 00:00:00</t>
+        </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -8755,7 +8920,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -8768,8 +8933,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|62|廠內
-LineScan平台|2023-08-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|62|Machine_084|2023-08-29</t>
         </is>
       </c>
     </row>
@@ -8845,7 +9009,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -8858,13 +9022,15 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|63|TTLM10009|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|63|Machine_085|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
-        <v>45460</v>
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2024-06-17 00:00:00</t>
+        </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -8919,7 +9085,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -8932,13 +9098,15 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|64|ASLM32002|2024-06-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|64|Machine_021|2024-06-17</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
-        <v>45526</v>
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2024-08-22 00:00:00</t>
+        </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -9010,7 +9178,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -9023,13 +9191,15 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|65|SSDM10001WSD|2024-08-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|65|Machine_086|2024-08-22</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
-        <v>45531</v>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2024-08-27 00:00:00</t>
+        </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -9097,7 +9267,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -9110,13 +9280,15 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|66|SSDM10001WSD|2024-08-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|66|Machine_086|2024-08-27</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
-        <v>45545</v>
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2024-09-10 00:00:00</t>
+        </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -9173,7 +9345,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -9186,13 +9358,15 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|67|SSDM10001WSD|2024-09-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|67|Machine_086|2024-09-10</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
-        <v>45668</v>
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2025-01-11 00:00:00</t>
+        </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -9256,7 +9430,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -9269,13 +9443,15 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|68|TTLM20008|2025-01-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|68|Machine_087|2025-01-11</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
-        <v>45702</v>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2025-02-14 00:00:00</t>
+        </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -9332,7 +9508,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -9345,13 +9521,15 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|69|SSLM21004SRA|2025-02-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|69|Machine_088|2025-02-14</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
-        <v>45902</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2025-09-02 00:00:00</t>
+        </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -9408,7 +9586,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -9421,13 +9599,15 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|70|SSLM21002SI|2025-09-02</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|70|Machine_089|2025-09-02</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
-        <v>45906</v>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2025-09-06 00:00:00</t>
+        </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -9502,7 +9682,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -9515,13 +9695,15 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|71|SSLM21003SI|2025-09-06</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|71|Machine_090|2025-09-06</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
-        <v>45933</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2025-10-03 00:00:00</t>
+        </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -9589,7 +9771,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -9602,13 +9784,15 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|72|SSLM21003SI|2025-10-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|72|Machine_090|2025-10-03</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
-        <v>45985</v>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2025-11-24 00:00:00</t>
+        </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -9666,7 +9850,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -9679,13 +9863,15 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|73|TTLM10015|2025-11-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|73|Machine_036|2025-11-24</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
-        <v>46008</v>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2025-12-17 00:00:00</t>
+        </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -9752,7 +9938,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -9765,13 +9951,15 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|74|ASLM32003|2025-12-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|74|Machine_091|2025-12-17</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
-        <v>46017</v>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2025-12-26 00:00:00</t>
+        </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -9836,7 +10024,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>廠內裝機問題</t>
+          <t>Internal_Dept裝機問題</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -9849,13 +10037,15 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠內裝機問題|75|ASLM32003|2025-12-26</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|Internal_Dept裝機問題|75|Machine_091|2025-12-26</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
-        <v>43449</v>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2018-12-15 00:00:00</t>
+        </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -9920,13 +10110,15 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|0|SSST20008TS|2018-12-15</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|0|Machine_092|2018-12-15</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
-        <v>43452</v>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2018-12-18 00:00:00</t>
+        </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -9997,13 +10189,15 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|1|SSST20008TS|2018-12-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|1|Machine_092|2018-12-18</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
-        <v>43562</v>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2019-04-07 00:00:00</t>
+        </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -10069,13 +10263,15 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|2|SSST20008TS|2019-04-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|2|Machine_092|2019-04-07</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
-        <v>43601</v>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2019-05-16 00:00:00</t>
+        </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10143,13 +10339,15 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|3|ASDM6109|2019-05-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|3|Machine_093|2019-05-16</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
-        <v>43528</v>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2019-03-04 00:00:00</t>
+        </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -10215,13 +10413,15 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|4|ASSH5105|2019-03-04</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|4|Machine_094|2019-03-04</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
-        <v>43728</v>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2019-09-20 00:00:00</t>
+        </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -10289,13 +10489,15 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|5|SSLM13005NR|2019-09-20</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|5|Machine_041|2019-09-20</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
-        <v>43751</v>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2019-10-13 00:00:00</t>
+        </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -10361,13 +10563,15 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|6|SSST11006|2019-10-13</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|6|Machine_095|2019-10-13</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
-        <v>43752</v>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2019-10-14 00:00:00</t>
+        </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -10435,13 +10639,15 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|7|SSLM10029|2019-10-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|7|Machine_096|2019-10-14</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
-        <v>43752</v>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2019-10-14 00:00:00</t>
+        </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -10509,13 +10715,15 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|8|ASDM6147|2019-10-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|8|Machine_097|2019-10-14</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
-        <v>43800</v>
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2019-12-01 00:00:00</t>
+        </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -10581,13 +10789,15 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|9|SSST20001TS|2019-12-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|9|Machine_098|2019-12-01</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
-        <v>43903</v>
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2020-03-13 00:00:00</t>
+        </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -10660,13 +10870,15 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|10|SSST20002TS|2020-03-13</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|10|Machine_099|2020-03-13</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
-        <v>43908</v>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2020-03-18 00:00:00</t>
+        </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -10731,13 +10943,15 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|11|PVOT0931|2020-03-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|11|Machine_100|2020-03-18</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
-        <v>43906</v>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2020-03-16 00:00:00</t>
+        </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -10803,13 +11017,15 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|12|SSST20002TS|2020-03-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|12|Machine_099|2020-03-16</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
-        <v>43937</v>
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2020-04-16 00:00:00</t>
+        </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -10878,13 +11094,15 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|13|SSLM10025|2020-04-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|13|Machine_101|2020-04-16</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
-        <v>43938</v>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2020-04-17 00:00:00</t>
+        </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10950,7 +11168,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|14|SSLM10025|2020-04-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|14|Machine_101|2020-04-17</t>
         </is>
       </c>
     </row>
@@ -11026,13 +11244,15 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|15|SSLM10025|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|15|Machine_101|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
-        <v>43974</v>
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2020-05-23 00:00:00</t>
+        </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -11100,13 +11320,15 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|16|SSLM21003NR|2020-05-23</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|16|Machine_017|2020-05-23</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
-        <v>43990</v>
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2020-06-08 00:00:00</t>
+        </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -11173,13 +11395,15 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|17|TTLM10008|2020-06-08</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|17|Machine_102|2020-06-08</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
-        <v>43987</v>
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2020-06-05 00:00:00</t>
+        </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -11250,13 +11474,15 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|18|ASDM5025|2020-06-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|18|Machine_103|2020-06-05</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
-        <v>43994</v>
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2020-06-12 00:00:00</t>
+        </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -11321,13 +11547,15 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|19|PVOT0931|2020-06-12</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|19|Machine_100|2020-06-12</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
-        <v>44010</v>
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2020-06-28 00:00:00</t>
+        </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -11397,13 +11625,15 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|20|SSST20007TS|2020-06-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|20|Machine_104|2020-06-28</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
-        <v>44010</v>
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2020-06-28 00:00:00</t>
+        </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -11477,13 +11707,15 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|21|SSST20003TS|2020-06-28</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|21|Machine_035|2020-06-28</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
-        <v>44075</v>
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2020-09-01 00:00:00</t>
+        </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -11547,13 +11779,15 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|22|BLMH2000|2020-09-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|22|Machine_105|2020-09-01</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
-        <v>44084</v>
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2020-09-10 00:00:00</t>
+        </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -11620,13 +11854,15 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|23|SSLM|2020-09-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|23|Machine_010|2020-09-10</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
-        <v>44140</v>
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2020-11-05 00:00:00</t>
+        </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -11692,13 +11928,15 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|24|SSLM(舊機)|2020-11-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|24|Machine_106|2020-11-05</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
-        <v>44159</v>
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2020-11-24 00:00:00</t>
+        </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -11772,13 +12010,15 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|25|ASDM6147|2020-11-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|25|Machine_097|2020-11-24</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
-        <v>44176</v>
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2020-12-11 00:00:00</t>
+        </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -11850,13 +12090,15 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|26|SSLM23001SR|2020-12-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|26|Machine_022|2020-12-11</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
-        <v>44265</v>
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2021-03-10 00:00:00</t>
+        </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -11922,13 +12164,15 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|27|SSLM21003SR|2021-03-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|27|Machine_107|2021-03-10</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
-        <v>44309</v>
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2021-04-23 00:00:00</t>
+        </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -11998,13 +12242,15 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|28|TTLM20001|2021-04-23</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|28|Machine_108|2021-04-23</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
-        <v>44337</v>
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2021-05-21 00:00:00</t>
+        </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -12072,13 +12318,15 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|29|SSLM21004SK|2021-05-21</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|29|Machine_046|2021-05-21</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
-        <v>44348</v>
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2021-06-01 00:00:00</t>
+        </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -12150,13 +12398,15 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|30|SSLM21004SK|2021-06-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|30|Machine_046|2021-06-01</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
-        <v>44442</v>
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2021-09-03 00:00:00</t>
+        </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -12222,13 +12472,15 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|31|SSST20002TS|2021-09-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|31|Machine_099|2021-09-03</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
-        <v>44457</v>
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2021-09-18 00:00:00</t>
+        </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -12295,7 +12547,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|32|SSST20001IC|2021-09-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|32|Machine_065|2021-09-18</t>
         </is>
       </c>
     </row>
@@ -12370,13 +12622,15 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|33|ASDM6147|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|33|Machine_097|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
-        <v>44293</v>
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2021-04-07 00:00:00</t>
+        </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -12445,7 +12699,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|34|ASDM6110|2021-04-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|34|Machine_109|2021-04-07</t>
         </is>
       </c>
     </row>
@@ -12532,13 +12786,15 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|35|SSST20003ZC|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|35|Machine_110|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
-        <v>44710</v>
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2022-05-29 00:00:00</t>
+        </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -12605,13 +12861,15 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|36|SSLM21016SR|2022-05-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|36|Machine_111|2022-05-29</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
-        <v>44714</v>
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2022-06-02 00:00:00</t>
+        </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -12680,13 +12938,15 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|37|ASDM6127|2022-06-02</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|37|Machine_112|2022-06-02</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
-        <v>44721</v>
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2022-06-09 00:00:00</t>
+        </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -12757,13 +13017,15 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|38|SSLM13011SR|2022-06-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|38|Machine_037|2022-06-09</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
-        <v>44714</v>
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2022-06-02 00:00:00</t>
+        </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -12827,13 +13089,15 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|39|SSLM21003SRNS|2022-06-02</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|39|Machine_113|2022-06-02</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
-        <v>44726</v>
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2022-06-14 00:00:00</t>
+        </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -12907,13 +13171,15 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|40|SSST30001WSD|2022-06-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|40|Machine_005|2022-06-14</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
-        <v>44860</v>
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2022-10-26 00:00:00</t>
+        </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -12978,13 +13244,15 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|41|SSLM-VAS|2022-10-26</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|41|Machine_114|2022-10-26</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
-        <v>44861</v>
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2022-10-27 00:00:00</t>
+        </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -13051,13 +13319,15 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|42|SSLM21010NR|2022-10-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|42|Machine_012|2022-10-27</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
-        <v>44874</v>
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2022-11-09 00:00:00</t>
+        </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -13132,13 +13402,15 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|43|SSLM21011NR|2022-11-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|43|Machine_019|2022-11-09</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
-        <v>44878</v>
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2022-11-13 00:00:00</t>
+        </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -13217,13 +13489,15 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|44|SSST30001WSD|2022-11-13</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|44|Machine_005|2022-11-13</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
-        <v>44964</v>
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2023-02-07 00:00:00</t>
+        </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -13292,13 +13566,15 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|45|SSLM21002SRC|2023-02-07</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|45|Machine_115|2023-02-07</t>
         </is>
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
-        <v>45027</v>
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2023-04-11 00:00:00</t>
+        </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -13379,14 +13655,15 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|46|SSST20006TS
-(2#)|2023-04-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|46|Machine_116|2023-04-11</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
-        <v>45062</v>
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2023-05-16 00:00:00</t>
+        </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -13458,7 +13735,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|47|SSLM21012SR|2023-05-16</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|47|Machine_013|2023-05-16</t>
         </is>
       </c>
     </row>
@@ -13540,13 +13817,15 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|48|SSST30003TS|UNKNOWN</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|48|Machine_073|UNKNOWN</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
-        <v>45070</v>
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2023-05-24 00:00:00</t>
+        </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -13636,13 +13915,15 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|49|SSST22001ZC|2023-05-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|49|Machine_040|2023-05-24</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
-        <v>45075</v>
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2023-05-29 00:00:00</t>
+        </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -13718,13 +13999,15 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|50|SSST30003TS|2023-05-29</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|50|Machine_073|2023-05-29</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
-        <v>45118</v>
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2023-07-11 00:00:00</t>
+        </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -13804,13 +14087,15 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|51|SSST30001WSD|2023-07-11</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|51|Machine_005|2023-07-11</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
-        <v>45148</v>
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2023-08-10 00:00:00</t>
+        </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -13887,13 +14172,15 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|52|SSLM25001NR|2023-08-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|52|Machine_031|2023-08-10</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
-        <v>45139</v>
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2023-08-01 00:00:00</t>
+        </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -13971,13 +14258,15 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|53|ASDM6140 |2023-08-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|53|Machine_117 |2023-08-01</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
-        <v>45155</v>
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2023-08-17 00:00:00</t>
+        </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -14053,13 +14342,15 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|54|SSST20008TS|2023-08-17</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|54|Machine_092|2023-08-17</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
-        <v>45156</v>
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2023-08-18 00:00:00</t>
+        </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -14155,13 +14446,15 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|55|SSST22001WCF|2023-08-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|55|Machine_118|2023-08-18</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
-        <v>45205</v>
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2023-10-06 00:00:00</t>
+        </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -14234,13 +14527,15 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|56|TTLM20001|2023-10-06</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|56|Machine_108|2023-10-06</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
-        <v>45217</v>
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2023-10-18 00:00:00</t>
+        </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -14315,13 +14610,15 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|57|SSLM11008NR|2023-10-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|57|Machine_119|2023-10-18</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
-        <v>45254</v>
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2023-11-24 00:00:00</t>
+        </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -14399,13 +14696,15 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|58|SSLM21019SR|2023-11-24</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|58|Machine_024|2023-11-24</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
-        <v>45257</v>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2023-11-27 00:00:00</t>
+        </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -14482,13 +14781,15 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|59|SSLM21003SRA|2023-11-27</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|59|Machine_004|2023-11-27</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
-        <v>45275</v>
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2023-12-15 00:00:00</t>
+        </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -14560,13 +14861,15 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|60|SSST11012|2023-12-15</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|60|Machine_120|2023-12-15</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
-        <v>45321</v>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2024-01-30 00:00:00</t>
+        </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -14634,13 +14937,15 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|61|SSLM23002LRS|2024-01-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|61|Machine_121|2024-01-30</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
-        <v>45365</v>
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2024-03-14 00:00:00</t>
+        </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -14712,13 +15017,15 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|62|ASDM6153|2024-03-14</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|62|Machine_122|2024-03-14</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
-        <v>45504</v>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2024-07-31 00:00:00</t>
+        </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -14784,13 +15091,15 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|63|ASDM6150|2024-07-31</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|63|Machine_123|2024-07-31</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
-        <v>45505</v>
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2024-08-01 00:00:00</t>
+        </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -14881,13 +15190,15 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|64|SSST20001WCF|2024-08-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|64|Machine_032|2024-08-01</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
-        <v>45547</v>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2024-09-12 00:00:00</t>
+        </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -14964,13 +15275,15 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|65|BLMH2004|2024-09-12</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|65|Machine_124|2024-09-12</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
-        <v>45595</v>
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2024-10-30 00:00:00</t>
+        </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -15043,13 +15356,15 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|66|SSST32003TC|2024-10-30</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|66|Machine_020|2024-10-30</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
-        <v>45691</v>
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2025-02-03 00:00:00</t>
+        </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -15129,13 +15444,15 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|67|TBPP14101|2025-02-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|67|Machine_125|2025-02-03</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
-        <v>45693</v>
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2025-02-05 00:00:00</t>
+        </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -15206,13 +15523,15 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|68|SSST22001WCF|2025-02-05</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|68|Machine_118|2025-02-05</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
-        <v>45720</v>
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2025-03-04 00:00:00</t>
+        </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -15280,13 +15599,15 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|69|TTLM20005|2025-03-04</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|69|Machine_126|2025-03-04</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
-        <v>45780</v>
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2025-05-03 00:00:00</t>
+        </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -15362,13 +15683,15 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|70|SSLM13003NR|2025-05-03</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|70|Machine_127|2025-05-03</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
-        <v>45797</v>
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2025-05-20 00:00:00</t>
+        </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -15458,13 +15781,15 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|71|SSLM21004SRA|2025-05-20</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|71|Machine_088|2025-05-20</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
-        <v>45816</v>
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2025-06-08 00:00:00</t>
+        </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -15541,13 +15866,15 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|72|SSLM21002SRA|2025-06-08</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|72|Machine_128|2025-06-08</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
-        <v>45861</v>
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2025-07-23 00:00:00</t>
+        </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -15627,13 +15954,15 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|73|TTLM20005|2025-07-23</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|73|Machine_126|2025-07-23</t>
         </is>
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
-        <v>45878</v>
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2025-08-09 00:00:00</t>
+        </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -15713,13 +16042,15 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|74|TTLM20004|2025-08-09</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|74|Machine_129|2025-08-09</t>
         </is>
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
-        <v>45879</v>
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2025-08-10 00:00:00</t>
+        </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -15790,13 +16121,15 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|75|TTLM10006|2025-08-10</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|75|Machine_130|2025-08-10</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
-        <v>45938</v>
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2025-10-08 00:00:00</t>
+        </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -15867,13 +16200,15 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|76|ASDM6149|2025-10-08</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|76|Machine_131|2025-10-08</t>
         </is>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
-        <v>45922</v>
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2025-09-22 00:00:00</t>
+        </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -15944,13 +16279,15 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|77|SSST20006TS |2025-09-22</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|77|Machine_132 |2025-09-22</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
-        <v>44487</v>
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2021-10-18 00:00:00</t>
+        </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -16027,13 +16364,15 @@
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|78|SSST11012|2021-10-18</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|78|Machine_120|2021-10-18</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
-        <v>45992</v>
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2025-12-01 00:00:00</t>
+        </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -16122,7 +16461,7 @@
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|79|SSST20010TC|2025-12-01</t>
+          <t>20251227-LineScan Strip機台軟硬體問題記錄.xlsx|廠外硬體損壞|79|Machine_133|2025-12-01</t>
         </is>
       </c>
     </row>

</xml_diff>